<commit_message>
ran the project once with test
</commit_message>
<xml_diff>
--- a/data/llm/first_pass/22_first_pass.xlsx
+++ b/data/llm/first_pass/22_first_pass.xlsx
@@ -454,7 +454,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>All candidates are identical to the reference item in material, dimensions, and function.</t>
+          <t>All candidates are identical to the reference item.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -472,7 +472,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>תוספת למחיצות גבס עבור לוח פח מגולוון בעובי 3 ממ המחובר לניצבים של המחיצה למניעת פריצה.</t>
+          <t>תוספת למחיצות גבס עבור לוח פח מגולוון בעubi 3 ממ המחובר לניצבים של המחיצה למניעת פריצה.</t>
         </is>
       </c>
       <c r="G2" t="b">
@@ -485,7 +485,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Candidates 0-1 match the fire-resistant gypsum board material and application context, while candidates 2-5 refer to partitions which is a different application.</t>
+          <t>All candidates are identical and match the reference for material and use.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -503,7 +503,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>תוספת מחיר ללוחות הגבס עבור שימוש בלוחות גבס חסין אש )וורוד(, בהתאם לתקן ולתכנית הבטיחות. המדידה לפי שטח נטו של הלוח חסין אש.</t>
+          <t>תוספת מחיר ללוחות הגבס עבור שימוש בלוחות גבס חassin אש )וורוד(, בהתאם לתקן ולתוכנית הבטיחות. המדידה לפי שטח נטו של הלוח חassin אש.</t>
         </is>
       </c>
       <c r="G3" t="b">
@@ -516,7 +516,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Candidates are for standard wall/ceiling drywall, not pipe enclosures with specific insulation and sealing requirements.</t>
+          <t>All candidates are identical and match the reference</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -524,11 +524,17 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>חיפוי פנים לקירות בלוח גבס, לרבות לוח גבס בעובי 12.5 ממ, קונסטרוקציה מפרופילי אומגה מחוזקת לקיר ו/או קונסטרוקציה עם מסילה עליונה ותחתונה וניצבים מפחפלדה מגולוון כל 40 סמ, כולל מזרני צמר סלעים בעובי 2 במשקל מרחבי 80 קג/מק. כולל שפכטל, הכל עד גמר מושלם מוכן לצביעה.</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>חיפוי/סגירה סביב צינורות בלוחות גבס דו-קרומי, לרבות קונסטרוקציה מפח מגולבן מכופף, מזרוני צמר זכוכית בעובי 3 במשקל מרחבי של 24קג/מק ואיטום בקוי המפגש עם משטחים צמודים כגון רצפות,קירות ותקרות, המדידה לפי שטח לוחות הגבס הנראים לעין.</t>
+          <t>חיפוי/סגירה סביב צינורות בלוחות גבס דו-קרומי, לרבות קונסטרוקציה מפח מגולבן מכופף, מזרוני צמר זכוכית בעובי 3במשקל מרחבי של 24קג/מק ואיטום בקוי המפגש עם משטחים צמודים כגון רצפות,קירות ותקרות, המדידה לפי שטח לוחות הגבס הנראים לעין.</t>
         </is>
       </c>
       <c r="G4" t="b">
@@ -541,7 +547,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Candidates 1-5 match material and dimensions but differ in stud spacing (30cm vs 40cm) and stud width (70mm vs unspecified), making them non-equivalent.</t>
+          <t>Matches material and dimensions closely.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -549,11 +555,17 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>מחיצות מסורגות על פי פרט חברת אורבונד מלוחות גבס דו-קרומי מכל צד בעובי כולל כ-12 סמ, לרבות קונסטרוקציה מפח מגולוון ברוחב 70 ממ, עם ניצבים כל 30 סמ,כולל מזרני צמר סלעים בעובי 2 במשקל מרחבי 80 קג/מק הכל עד גמר מושלם, כולל שפכטל, מוכן לצביעה. המדידה נטו ללא פתחים.</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>מחיצות גבס דו קרומיות ) 2פלטות בכל צד- עובי 12.5ממ (בעובי כולל של 120ממ לרבות מסלול עליון ותחתון מפח מגוולון וניצבים כל 40סמ )עובי 0.8ממ (,צמרסלעים בעובי 2לבידוד משקל מרחבי 80קג / מק , כולל שפכטל גמר מוכן לצבע, קומפלט. ) פתחים לא ימדדו בשטח הכללי וינוכו שטחם אם כי יצירת הפתחים כלולה ב</t>
+          <t>מחיצות גבס דו קרומיות ) 2פלטות בכל צד- עobi 12.5ממ (בעobi כולל של 120ממ לרבות מסלול עליון ותחתון מפח מגוולון וניצבים כל 40סמ )עobi 0.8ממ (,צמרסלעים בעobi 2לבידוד משקל מרחבי 80קג / מק , כולל שפכטל גמר מוכן לצבע, קומפלט. ) פתחים לא ימדדו בשטח הכללי וינוכו שטחם אם כי יצירת הפתחים כלולה ב</t>
         </is>
       </c>
       <c r="G5" t="b">
@@ -566,7 +578,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Candidate 5 matches the reference material (double-layer gypsum board, galvanized steel framing) and intended use (interior cladding), while others differ in specific application or material.</t>
+          <t>Best match based on material and dimensions.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -575,11 +587,11 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>חיפוי פנים לקירות בלוח גבס, לרבות לוח גבס בעובי 12.5 ממ, קונסטרוקציה מפרופילי אומגה מחוזקת לקיר ו/או קונסטרוקציה עם מסילה עליונה ותחתונה וניצבים מפחפלדה מגולוון כל 40 סמ, כולל מזרני צמר סלעים בעובי 2 במשקל מרחבי 80 קג/מק. כולל שפכטל, הכל עד גמר מושלם מוכן לצביעה.</t>
+          <t>תוספת למחיצת גבס דו-קרומיות עבור בניה וחיזוק פתח מניצבי פח ברוחב 5 סמ ובעובי 0.8-1.25 ממ, לביצוע כיס, לדלת הזזה לתוך כיס לרבות חיזוק משקוף הדלת (משקוף ודלת נמדדים בנפרד)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -597,7 +609,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Material mismatch: reference is perforated steel, candidates are unperforated galvanized steel.</t>
+          <t>Material and dimensions match reference</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -605,11 +617,17 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>תקרה דגם C - תקרת מגשי פח מגולוון וצבוע. מגשים לא מחוררים, ברוחב 30 סמ ובעובי 0.6 ממ - המחיר כולל את הפרופילים הנושאים, אלמנטי התליה, וגמר פרופילי Z+L היקפיים, לרבות פרופיל אומגה בין השדות, אם נדרש.</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>תקרת מגשי פח מחורר , ניקוב עגול, עובי 0.8ממ ברוחב 30סמ בסוג וגוון בהתאם לרשימת גמרים מצורפת של לאומית - הבצוע כולל גם קונסטרוקציה וחיזוקים עפי הLZ צורך כולל זויתני</t>
+          <t>תקרת מגשי פח מחורר , ניקוב עגול, עobi 0.8ממ ברוחב 30סמ בסוג וגוון בהתאם לרשימת גמרים מצורפת של לאומית - הבצוע כולל גם קונסטרוקציה וחיזוקים עפי הLZ צורך כולל זויתני</t>
         </is>
       </c>
       <c r="G7" t="b">
@@ -622,7 +640,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Candidates 2-5 match the reference material (ECOPHON-FOCUS-A) and dimensions (60/60 cm), while candidates 0-1 are different materials.</t>
+          <t>Matches material and dimensions with high confidence.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -640,7 +658,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>תקרת אריחי תקרה אקוסטית דוגמת  FOCUS Aשל אקופון או שע במידות 60/60סמ ת בסוג וגוון עפי האדריכל - הבצוע . LZכולל גם קונסטרוקציה וחיזוקים עפי הצוLZ רך כולל זויתני</t>
+          <t>תקרת אריחי תקרה אקוסטית דוגמת FOCUS Aשל אקופון או שע במידות 60/60סמ ת בסוג וגוון עפי האדריכל - הבצוע . LZכולל גם קונסטרוקציה וחיזוקים עפי הצוLZ רך כולל זויתני</t>
         </is>
       </c>
       <c r="G8" t="b">
@@ -653,7 +671,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Candidates 0-2 match the reference material and application (drywall reinforcement), while candidates 3-5 describe wall cladding.</t>
+          <t>All candidates are identical and match the reference material.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -671,7 +689,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>חיזוקים בקירות גבס ככול שנדרש לפי תכנית )כיור שוקת, כיור שירותים, מאחז יד נכים, מסכ(</t>
+          <t>חיזוקים בקירות גבס ככול שנדרש לפי תכנית )כיור שוקת, כיור שירותים, מאחז יד נכים, מסכים(</t>
         </is>
       </c>
       <c r="G9" t="b">
@@ -684,7 +702,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Candidates 0, 1, and 5 match the material (gypsum board ceiling) and dimensions (12.7 mm), while candidates 2, 3, and 4 describe different applications or materials.</t>
+          <t>Best match based on material and dimensions.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -715,7 +733,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>No candidate matches the reference item as it specifies a specific application (complete door frames) while all candidates are for fire doors or heavy doors.</t>
+          <t>All candidates match reference exactly.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -723,8 +741,14 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>חיזוק אנכי למשקוף עבור דלת אש או דלת כבדה במחיצות גבס עי פרופיל פלדה מגולוון 70/70/2.6 ממ, לרבות עיגון לרצפה ולתקרת הבטון על ידי פלטקה ו-4 ברגי עיגון.</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>חיזוקים ופרופיל מחוזק או RHSבמשקופי דלתות קומפלט לדלת עפי הנחיות אורבונד</t>
@@ -740,7 +764,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Candidate 3 matches the reference item as it describes ceiling and ceiling grid gypsum board with 12.7mm thickness, matching the reference's dimensions and material.</t>
+          <t>Matches material and dimensions for gypsonboard walls.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -748,8 +772,14 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>מחיצות מסורגות על פי פרט חברת אורבונד מלוחות גבס דו-קרומי מכל צד בעובי כולל כ-12 סמ, לרבות קונסטרוקציה מפח מגולוון ברוחב 70 ממ, עם ניצבים כל 30 סמ,כולל מזרני צמר סלעים בעובי 2 במשקל מרחבי 80 קג/מק הכל עד גמר מושלם, כולל שפכטל, מוכן לצביעה. המדידה נטו ללא פתחים.</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>סינר גבס אופקי ואנכי במידות שונות בגבהים שונים עפי התוכניות בפריסה לרבות כל קונסטרקציית העזר הנדרשת גמר שפכטל מוכן לצבע כולל פינות מגן ובמידות שונות. הבצוע כולל גם הכנות לתאורה נסתרת ,</t>
@@ -765,7 +795,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Material mismatch: reference is gypsum board coving, candidates are lead sheets or other gypsum board items.</t>
+          <t>Best match based on material and dimensions.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -773,8 +803,14 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>תוספת למחיצות גבס עבור חיפוי פנימי ביריעות עופרת נגד קרינה בעובי 1.5 ממ. לרבות חפיפה של 2-5 סמ ואטימת הברגים. היריעה בגליל ברוחב 1.0 מטר ואורך 2.9 מטר, דוגמת א.א. מ.פ.ה או שע. (חדר צילום רנטגן)</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
           <t>קרניז תאורה בחתך של כ- 35/15סמ מלוחות גבס לרבות חלקים אופקיים ואנכיים, קונסטרוקצית תליה וחיזוק, מגיני פינות והחיזוקים הדרושים לחיבור גוף התאורה, המדידה לפי אורך הקרניז על כל חלקיו.</t>

</xml_diff>